<commit_message>
Catálogo real: 63 productos del chat de WhatsApp, placeholder para prendas sin foto
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/aika.xlsx
+++ b/data/aika.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M64"/>
   <cols>
     <col min="1" max="1" width="7.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -460,28 +460,28 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>EN01</v>
+        <v>CS01</v>
       </c>
       <c r="B2" t="str">
-        <v>Enterito Suplex</v>
+        <v>Catsuit Curve</v>
       </c>
       <c r="C2" t="str">
-        <v>Enteritos</v>
+        <v>Bodys y catsuits</v>
       </c>
       <c r="D2" t="str">
         <v>Mujer</v>
       </c>
       <c r="E2">
-        <v>32900</v>
+        <v>24000</v>
       </c>
       <c r="F2" t="str">
         <v/>
       </c>
       <c r="G2">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="H2" t="str">
-        <v>S,M,L</v>
+        <v>S/M (38/40),L/XL (42/44)</v>
       </c>
       <c r="I2" t="str">
         <v>rosa,bordo,rosa claro,gris azulado,azul marino,verde,negro,azul,celeste</v>
@@ -496,80 +496,80 @@
         <v>si</v>
       </c>
       <c r="M2" t="str">
-        <v>Suplex elastizado, tiras regulables, tazas desmontables y costuras que definen.</v>
+        <v>Suplex elastizado, tiras regulables y tazas desmontables.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>TO01</v>
+        <v>CS02</v>
       </c>
       <c r="B3" t="str">
-        <v>Musculosa Melville Puntilla</v>
+        <v>Catsuit Algodón Lycra</v>
       </c>
       <c r="C3" t="str">
-        <v>Tops</v>
+        <v>Bodys y catsuits</v>
       </c>
       <c r="D3" t="str">
         <v>Mujer</v>
       </c>
       <c r="E3">
-        <v>15900</v>
+        <v>18000</v>
       </c>
       <c r="F3" t="str">
         <v/>
       </c>
       <c r="G3">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="H3" t="str">
-        <v>S,M,L</v>
+        <v>Único</v>
       </c>
       <c r="I3" t="str">
-        <v>blanco,negro</v>
+        <v>negro,gris,blanco,chocolate,rosa,azul,rojo</v>
       </c>
       <c r="J3" t="str">
-        <v>aika-05.jpg,aika-08.jpg</v>
+        <v/>
       </c>
       <c r="K3" t="str">
-        <v>si</v>
+        <v>no</v>
       </c>
       <c r="L3" t="str">
         <v>no</v>
       </c>
       <c r="M3" t="str">
-        <v>Tela melville de verano con detalle de puntilla en el borde.</v>
+        <v>Algodón lycra premium. Talle único, cede a un M.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>TO02</v>
+        <v>CS03</v>
       </c>
       <c r="B4" t="str">
-        <v>Musculosa Morley Básica</v>
+        <v>Catsuit Forrado Soft</v>
       </c>
       <c r="C4" t="str">
-        <v>Tops</v>
+        <v>Bodys y catsuits</v>
       </c>
       <c r="D4" t="str">
         <v>Mujer</v>
       </c>
       <c r="E4">
-        <v>11900</v>
+        <v>18500</v>
       </c>
       <c r="F4" t="str">
         <v/>
       </c>
       <c r="G4">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="H4" t="str">
-        <v>Único</v>
+        <v>S (38/40),L (40/42)</v>
       </c>
       <c r="I4" t="str">
-        <v>negro,topo,chocolate,blanco,gris</v>
+        <v>negro</v>
       </c>
       <c r="J4" t="str">
-        <v>aika-01.jpg</v>
+        <v/>
       </c>
       <c r="K4" t="str">
         <v>no</v>
@@ -578,39 +578,39 @@
         <v>no</v>
       </c>
       <c r="M4" t="str">
-        <v>Morley acanalado, calce al cuerpo. Un básico en cinco colores.</v>
+        <v>Modal soft, todo forrado (doble tela).</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>TO03</v>
+        <v>BO01</v>
       </c>
       <c r="B5" t="str">
-        <v>Musculosa de Tiras</v>
+        <v>Body Cadenas</v>
       </c>
       <c r="C5" t="str">
-        <v>Tops</v>
+        <v>Bodys y catsuits</v>
       </c>
       <c r="D5" t="str">
         <v>Mujer</v>
       </c>
       <c r="E5">
-        <v>12900</v>
-      </c>
-      <c r="F5">
-        <v>14900</v>
+        <v>16500</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
       </c>
       <c r="G5">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H5" t="str">
         <v>Único</v>
       </c>
       <c r="I5" t="str">
-        <v>chocolate,blanco,negro</v>
+        <v>negro</v>
       </c>
       <c r="J5" t="str">
-        <v>aika-02.jpg</v>
+        <v/>
       </c>
       <c r="K5" t="str">
         <v>no</v>
@@ -619,39 +619,39 @@
         <v>no</v>
       </c>
       <c r="M5" t="str">
-        <v>Tiritas finas y escote redondo, ideal para combinar.</v>
+        <v>Body con detalle de cadenas.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>TO04</v>
+        <v>BO02</v>
       </c>
       <c r="B6" t="str">
-        <v>Musculosa Rayada</v>
+        <v>Body Encaje Lencero</v>
       </c>
       <c r="C6" t="str">
-        <v>Tops</v>
+        <v>Bodys y catsuits</v>
       </c>
       <c r="D6" t="str">
         <v>Mujer</v>
       </c>
       <c r="E6">
-        <v>14900</v>
+        <v>16500</v>
       </c>
       <c r="F6" t="str">
         <v/>
       </c>
       <c r="G6">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="H6" t="str">
         <v>Único</v>
       </c>
       <c r="I6" t="str">
-        <v>celeste,rosa</v>
+        <v>negro</v>
       </c>
       <c r="J6" t="str">
-        <v>aika-03.jpg</v>
+        <v/>
       </c>
       <c r="K6" t="str">
         <v>no</v>
@@ -660,121 +660,121 @@
         <v>si</v>
       </c>
       <c r="M6" t="str">
-        <v>Tejido rayado con vivos de color en escote y sisas.</v>
+        <v>Encaje lencero, busto forrado. Talle único, aprox. S/M.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>PA01</v>
+        <v>BO03</v>
       </c>
       <c r="B7" t="str">
-        <v>Oxford Línea</v>
+        <v>Body Puntilla Espalda</v>
       </c>
       <c r="C7" t="str">
-        <v>Pantalones</v>
+        <v>Bodys y catsuits</v>
       </c>
       <c r="D7" t="str">
         <v>Mujer</v>
       </c>
       <c r="E7">
-        <v>27900</v>
+        <v>16000</v>
       </c>
       <c r="F7" t="str">
         <v/>
       </c>
       <c r="G7">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H7" t="str">
-        <v>S,M,L</v>
+        <v>Único</v>
       </c>
       <c r="I7" t="str">
         <v>negro</v>
       </c>
       <c r="J7" t="str">
-        <v>aika-09.jpg</v>
+        <v/>
       </c>
       <c r="K7" t="str">
-        <v>si</v>
+        <v>no</v>
       </c>
       <c r="L7" t="str">
         <v>no</v>
       </c>
       <c r="M7" t="str">
-        <v>Lycra importada, cintura en V y doble línea al costado.</v>
+        <v>Microfibra, busto forrado, con broche. Talle único, cede a un M.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>PA02</v>
+        <v>BO04</v>
       </c>
       <c r="B8" t="str">
-        <v>Jogger Wide Leg Batik</v>
+        <v>Body Cruzado Espalda</v>
       </c>
       <c r="C8" t="str">
-        <v>Pantalones</v>
+        <v>Bodys y catsuits</v>
       </c>
       <c r="D8" t="str">
         <v>Mujer</v>
       </c>
       <c r="E8">
-        <v>29900</v>
+        <v>15500</v>
       </c>
       <c r="F8" t="str">
         <v/>
       </c>
       <c r="G8">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H8" t="str">
-        <v>S,M,L</v>
+        <v>Único</v>
       </c>
       <c r="I8" t="str">
-        <v>gris</v>
+        <v>negro</v>
       </c>
       <c r="J8" t="str">
-        <v>aika-04.jpg</v>
+        <v/>
       </c>
       <c r="K8" t="str">
         <v>no</v>
       </c>
       <c r="L8" t="str">
-        <v>si</v>
+        <v>no</v>
       </c>
       <c r="M8" t="str">
-        <v>Tela rústica batik, bolsillos laterales y tanca ajustable.</v>
+        <v>Microfibra, busto forrado, con broche. Talle único, aprox. S.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>SH01</v>
+        <v>TP01</v>
       </c>
       <c r="B9" t="str">
-        <v>Short Sastrero con Cinto</v>
+        <v>Top Lucy Morley</v>
       </c>
       <c r="C9" t="str">
-        <v>Shorts</v>
+        <v>Tops</v>
       </c>
       <c r="D9" t="str">
         <v>Mujer</v>
       </c>
       <c r="E9">
-        <v>24900</v>
-      </c>
-      <c r="F9">
-        <v>29900</v>
+        <v>12000</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
       </c>
       <c r="G9">
         <v>10</v>
       </c>
       <c r="H9" t="str">
-        <v>S,M,L</v>
+        <v>Único</v>
       </c>
       <c r="I9" t="str">
-        <v>chocolate,negro,camel</v>
+        <v>negro,topo,gris,blanco,chocolate</v>
       </c>
       <c r="J9" t="str">
-        <v>aika-07.jpg</v>
+        <v>aika-01.jpg</v>
       </c>
       <c r="K9" t="str">
         <v>si</v>
@@ -783,60 +783,2274 @@
         <v>no</v>
       </c>
       <c r="M9" t="str">
-        <v>Tiro alto con cinto forrado. Va con todo.</v>
+        <v>Morley de algodón premium. Talle único, cede a M.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
+        <v>TP02</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Top Gigi Forrado</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Tops</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E10">
+        <v>12000</v>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10">
+        <v>10</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I10" t="str">
+        <v>negro,blanco,chocolate</v>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v>no</v>
+      </c>
+      <c r="L10" t="str">
+        <v>si</v>
+      </c>
+      <c r="M10" t="str">
+        <v>Microfibra premium, todo forrado (doble tela). Talle único, cede a M.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>TP03</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Top Algodón Lycra</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Tops</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E11">
+        <v>11000</v>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11">
+        <v>10</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I11" t="str">
+        <v>negro,blanco,celeste,chocolate,gris</v>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v>no</v>
+      </c>
+      <c r="L11" t="str">
+        <v>no</v>
+      </c>
+      <c r="M11" t="str">
+        <v>Algodón lycra premium. Talle único, cede a un M.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>TP04</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Corset Encaje Microfibra</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Tops</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E12">
+        <v>16500</v>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12">
+        <v>10</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I12" t="str">
+        <v>negro,blanco,chocolate</v>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v>no</v>
+      </c>
+      <c r="L12" t="str">
+        <v>no</v>
+      </c>
+      <c r="M12" t="str">
+        <v>Microfibra con detalle de encaje, delantera forrada. Base crop. Talle único, cede a un M.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>TP05</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Top Hillary Corset</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Tops</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E13">
+        <v>16500</v>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13">
+        <v>10</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I13" t="str">
+        <v>negro,blanco</v>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v>no</v>
+      </c>
+      <c r="L13" t="str">
+        <v>no</v>
+      </c>
+      <c r="M13" t="str">
+        <v>Encaje cassia elastizado, busto forrado. Talle único, cede a M.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>TP06</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Top Micro Lola</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Tops</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E14">
+        <v>14500</v>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14">
+        <v>10</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I14" t="str">
+        <v>blanco,negro,chocolate</v>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v>no</v>
+      </c>
+      <c r="L14" t="str">
+        <v>no</v>
+      </c>
+      <c r="M14" t="str">
+        <v>Microfibra con corpiño de encaje, busto forrado. Base crop. Talle único.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>TP07</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Corpiño Forrado Encaje</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Tops</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E15">
+        <v>13000</v>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15">
+        <v>10</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I15" t="str">
+        <v>negro,chocolate,blanco</v>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v>no</v>
+      </c>
+      <c r="L15" t="str">
+        <v>no</v>
+      </c>
+      <c r="M15" t="str">
+        <v>Encaje forrado de modal soft. Talle único.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>TP08</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Camisa Noa Encaje</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Tops</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E16">
+        <v>19000</v>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16">
+        <v>10</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I16" t="str">
+        <v>negro</v>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v>si</v>
+      </c>
+      <c r="L16" t="str">
+        <v>si</v>
+      </c>
+      <c r="M16" t="str">
+        <v>Encaje elastizado, botones funcionales. Base crop. Talle único, abarca M.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>MU01</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Musculosa Encanto</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Musculosas</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E17">
+        <v>15000</v>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17">
+        <v>10</v>
+      </c>
+      <c r="H17" t="str">
+        <v>2,3,4,5</v>
+      </c>
+      <c r="I17" t="str">
+        <v>blanco,negro,gris,rosa claro,celeste,marron</v>
+      </c>
+      <c r="J17" t="str">
+        <v>aika-05.jpg</v>
+      </c>
+      <c r="K17" t="str">
+        <v>si</v>
+      </c>
+      <c r="L17" t="str">
+        <v>no</v>
+      </c>
+      <c r="M17" t="str">
+        <v>Tela melville de verano.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>MU02</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Musculosa Renda</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Musculosas</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E18">
+        <v>15000</v>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18">
+        <v>10</v>
+      </c>
+      <c r="H18" t="str">
+        <v>2,3,4,5,6</v>
+      </c>
+      <c r="I18" t="str">
+        <v>rosa,gris,negro,blanco,marron</v>
+      </c>
+      <c r="J18" t="str">
+        <v>aika-08.jpg</v>
+      </c>
+      <c r="K18" t="str">
+        <v>no</v>
+      </c>
+      <c r="L18" t="str">
+        <v>no</v>
+      </c>
+      <c r="M18" t="str">
+        <v>Tela melville, larguitas, con puntilla en cuello y sisas.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>MU03</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Musculosa Ameli Morley</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Musculosas</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E19">
+        <v>14300</v>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19">
+        <v>10</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I19" t="str">
+        <v>chocolate,blanco,negro</v>
+      </c>
+      <c r="J19" t="str">
+        <v>aika-02.jpg</v>
+      </c>
+      <c r="K19" t="str">
+        <v>no</v>
+      </c>
+      <c r="L19" t="str">
+        <v>no</v>
+      </c>
+      <c r="M19" t="str">
+        <v>Morley de algodón premium. Son cortas. Talle único, cede a M.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>MU04</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Musculosa Rayada Hilo</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Musculosas</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E20">
+        <v>20000</v>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20">
+        <v>10</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I20" t="str">
+        <v>celeste,rosa</v>
+      </c>
+      <c r="J20" t="str">
+        <v>aika-03.jpg</v>
+      </c>
+      <c r="K20" t="str">
+        <v>no</v>
+      </c>
+      <c r="L20" t="str">
+        <v>si</v>
+      </c>
+      <c r="M20" t="str">
+        <v>Hilo lycra premium. Base crop. Talle único.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>MU05</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Musculosa Marni Puntilla</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Musculosas</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E21">
+        <v>15500</v>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21">
+        <v>10</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I21" t="str">
+        <v>chocolate,negro</v>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
+        <v>no</v>
+      </c>
+      <c r="L21" t="str">
+        <v>no</v>
+      </c>
+      <c r="M21" t="str">
+        <v>Marni con detalle de puntilla. Base crop. Talle único, cede a un M.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>MU06</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Musculosa Kenia Botón</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Musculosas</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E22">
+        <v>28500</v>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22">
+        <v>10</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I22" t="str">
+        <v>negro</v>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22" t="str">
+        <v>no</v>
+      </c>
+      <c r="L22" t="str">
+        <v>no</v>
+      </c>
+      <c r="M22" t="str">
+        <v>Importada. Hilo lycra premium, botones funcionales. Base clásica. Talle único, aprox. M.</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>MU07</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Musculosa Buche Morley</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Musculosas</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E23">
+        <v>14400</v>
+      </c>
+      <c r="F23" t="str">
+        <v/>
+      </c>
+      <c r="G23">
+        <v>10</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I23" t="str">
+        <v>negro,blanco,chocolate</v>
+      </c>
+      <c r="J23" t="str">
+        <v/>
+      </c>
+      <c r="K23" t="str">
+        <v>no</v>
+      </c>
+      <c r="L23" t="str">
+        <v>no</v>
+      </c>
+      <c r="M23" t="str">
+        <v>Morley tao con detalle de mostacillas. Talle único, aprox. M.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>MU08</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Musculosa Bretel Forrada</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Musculosas</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E24">
+        <v>12000</v>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+      <c r="G24">
+        <v>10</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I24" t="str">
+        <v>frambuesa,blanco,chocolate,negro</v>
+      </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+      <c r="K24" t="str">
+        <v>no</v>
+      </c>
+      <c r="L24" t="str">
+        <v>no</v>
+      </c>
+      <c r="M24" t="str">
+        <v>Modal soft, todo forrado (doble tela). Talle único, cede a un M.</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>RE01</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Remera Espejo</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Remeras</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E25">
+        <v>12500</v>
+      </c>
+      <c r="F25" t="str">
+        <v/>
+      </c>
+      <c r="G25">
+        <v>10</v>
+      </c>
+      <c r="H25" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I25" t="str">
+        <v>negro</v>
+      </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
+      <c r="K25" t="str">
+        <v>no</v>
+      </c>
+      <c r="L25" t="str">
+        <v>no</v>
+      </c>
+      <c r="M25" t="str">
+        <v>Tela melvin. Talle único hasta un L.</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>RE02</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Remera Pez</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Remeras</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E26">
+        <v>12000</v>
+      </c>
+      <c r="F26" t="str">
+        <v/>
+      </c>
+      <c r="G26">
+        <v>10</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I26" t="str">
+        <v>negro</v>
+      </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+      <c r="K26" t="str">
+        <v>no</v>
+      </c>
+      <c r="L26" t="str">
+        <v>no</v>
+      </c>
+      <c r="M26" t="str">
+        <v>Tela melvin. Talle único hasta un L.</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>RE03</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Remera NY Taxi</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Remeras</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E27">
+        <v>14500</v>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27">
+        <v>10</v>
+      </c>
+      <c r="H27" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I27" t="str">
+        <v>chocolate,blanco,negro,bordo</v>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+      <c r="K27" t="str">
+        <v>si</v>
+      </c>
+      <c r="L27" t="str">
+        <v>si</v>
+      </c>
+      <c r="M27" t="str">
+        <v>Algodón jersey, estampado DTF. Talle único, aprox. M/L.</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>RE04</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Remera Samara Cropped</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Remeras</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E28">
+        <v>13500</v>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28">
+        <v>10</v>
+      </c>
+      <c r="H28" t="str">
+        <v>S,L</v>
+      </c>
+      <c r="I28" t="str">
+        <v>negro,blanco,topo,chocolate,marron</v>
+      </c>
+      <c r="J28" t="str">
+        <v/>
+      </c>
+      <c r="K28" t="str">
+        <v>no</v>
+      </c>
+      <c r="L28" t="str">
+        <v>no</v>
+      </c>
+      <c r="M28" t="str">
+        <v>Algodón, modelo over boxy. S: sisa 50 cm, largo 50 cm. L: 57 x 57 cm.</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>RE05</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Camiseta Roma Encaje</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Remeras</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E29">
+        <v>16500</v>
+      </c>
+      <c r="F29" t="str">
+        <v/>
+      </c>
+      <c r="G29">
+        <v>10</v>
+      </c>
+      <c r="H29" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I29" t="str">
+        <v>chocolate,blanco,negro</v>
+      </c>
+      <c r="J29" t="str">
+        <v/>
+      </c>
+      <c r="K29" t="str">
+        <v>no</v>
+      </c>
+      <c r="L29" t="str">
+        <v>si</v>
+      </c>
+      <c r="M29" t="str">
+        <v>Encaje, manga con abertura. Pupera. Talle único, cede a M.</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>RE06</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Puperón Oversize</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Remeras</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E30">
+        <v>13000</v>
+      </c>
+      <c r="F30" t="str">
+        <v/>
+      </c>
+      <c r="G30">
+        <v>10</v>
+      </c>
+      <c r="H30" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I30" t="str">
+        <v>negro,blanco,chocolate</v>
+      </c>
+      <c r="J30" t="str">
+        <v/>
+      </c>
+      <c r="K30" t="str">
+        <v>no</v>
+      </c>
+      <c r="L30" t="str">
+        <v>no</v>
+      </c>
+      <c r="M30" t="str">
+        <v>Algodón, modelo oversize. Talle único, aprox. L/XL de sisa.</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>RE07</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Reme Top Algodón Lycra</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Remeras</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E31">
+        <v>14500</v>
+      </c>
+      <c r="F31" t="str">
+        <v/>
+      </c>
+      <c r="G31">
+        <v>10</v>
+      </c>
+      <c r="H31" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I31" t="str">
+        <v>negro,gris,blanco,chocolate</v>
+      </c>
+      <c r="J31" t="str">
+        <v/>
+      </c>
+      <c r="K31" t="str">
+        <v>no</v>
+      </c>
+      <c r="L31" t="str">
+        <v>no</v>
+      </c>
+      <c r="M31" t="str">
+        <v>Algodón lycra premium. Talle único, cede a M.</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>RE08</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Reme Brooklyn Crop</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Remeras</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E32">
+        <v>15500</v>
+      </c>
+      <c r="F32" t="str">
+        <v/>
+      </c>
+      <c r="G32">
+        <v>10</v>
+      </c>
+      <c r="H32" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I32" t="str">
+        <v>azul,negro,chocolate,rojo</v>
+      </c>
+      <c r="J32" t="str">
+        <v/>
+      </c>
+      <c r="K32" t="str">
+        <v>no</v>
+      </c>
+      <c r="L32" t="str">
+        <v>si</v>
+      </c>
+      <c r="M32" t="str">
+        <v>Algodón lycra estampado. Base crop. Talle único, cede a un M.</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>RE09</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Remera Boxy Rayada</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Remeras</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E33">
+        <v>17500</v>
+      </c>
+      <c r="F33" t="str">
+        <v/>
+      </c>
+      <c r="G33">
+        <v>10</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I33" t="str">
+        <v>blanco</v>
+      </c>
+      <c r="J33" t="str">
+        <v/>
+      </c>
+      <c r="K33" t="str">
+        <v>no</v>
+      </c>
+      <c r="L33" t="str">
+        <v>si</v>
+      </c>
+      <c r="M33" t="str">
+        <v>Algodón jersey premium, bordado. Modelo over, talle único (abarca aprox. L).</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>RE10</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Reme Tokio Puntilla</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Remeras</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E34">
+        <v>15000</v>
+      </c>
+      <c r="F34" t="str">
+        <v/>
+      </c>
+      <c r="G34">
+        <v>10</v>
+      </c>
+      <c r="H34" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I34" t="str">
+        <v>negro</v>
+      </c>
+      <c r="J34" t="str">
+        <v/>
+      </c>
+      <c r="K34" t="str">
+        <v>no</v>
+      </c>
+      <c r="L34" t="str">
+        <v>no</v>
+      </c>
+      <c r="M34" t="str">
+        <v>Microfibra, base crop (cortas). Talle único, cede a un M.</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>RE11</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Remera Micro Corset</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Remeras</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E35">
+        <v>17500</v>
+      </c>
+      <c r="F35" t="str">
+        <v/>
+      </c>
+      <c r="G35">
+        <v>10</v>
+      </c>
+      <c r="H35" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I35" t="str">
+        <v>chocolate,blanco,negro</v>
+      </c>
+      <c r="J35" t="str">
+        <v/>
+      </c>
+      <c r="K35" t="str">
+        <v>no</v>
+      </c>
+      <c r="L35" t="str">
+        <v>no</v>
+      </c>
+      <c r="M35" t="str">
+        <v>Microfibra, base crop. Talle único, cede a un M.</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>RE12</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Remera Virginia</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Remeras</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E36">
+        <v>16000</v>
+      </c>
+      <c r="F36" t="str">
+        <v/>
+      </c>
+      <c r="G36">
+        <v>10</v>
+      </c>
+      <c r="H36" t="str">
+        <v>2,3,4,5</v>
+      </c>
+      <c r="I36" t="str">
+        <v>crudo,negro,beige,azul,verde</v>
+      </c>
+      <c r="J36" t="str">
+        <v/>
+      </c>
+      <c r="K36" t="str">
+        <v>no</v>
+      </c>
+      <c r="L36" t="str">
+        <v>no</v>
+      </c>
+      <c r="M36" t="str">
+        <v>Melville (algodón con lycra de verano). Talle 2 en todos los colores; 3: natural, negro, beige, azul, verde; 4: natural, negro, beige; 5: natural, negro, verde. Sin cambio.</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
         <v>VE01</v>
       </c>
-      <c r="B10" t="str">
-        <v>Vestido Calado</v>
-      </c>
-      <c r="C10" t="str">
+      <c r="B37" t="str">
+        <v>Vestido Playero</v>
+      </c>
+      <c r="C37" t="str">
         <v>Vestidos</v>
       </c>
-      <c r="D10" t="str">
-        <v>Mujer</v>
-      </c>
-      <c r="E10">
-        <v>34900</v>
-      </c>
-      <c r="F10" t="str">
-        <v/>
-      </c>
-      <c r="G10">
-        <v>0</v>
-      </c>
-      <c r="H10" t="str">
-        <v>Único</v>
-      </c>
-      <c r="I10" t="str">
+      <c r="D37" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E37">
+        <v>19500</v>
+      </c>
+      <c r="F37" t="str">
+        <v/>
+      </c>
+      <c r="G37">
+        <v>10</v>
+      </c>
+      <c r="H37" t="str">
+        <v>Único (hasta XL)</v>
+      </c>
+      <c r="I37" t="str">
         <v>crudo,chocolate,blanco,negro</v>
       </c>
-      <c r="J10" t="str">
+      <c r="J37" t="str">
         <v>aika-06.jpg</v>
       </c>
-      <c r="K10" t="str">
-        <v>no</v>
-      </c>
-      <c r="L10" t="str">
-        <v>no</v>
-      </c>
-      <c r="M10" t="str">
-        <v>Tejido calado, manga larga y escote en V. También como salida de playa.</v>
+      <c r="K37" t="str">
+        <v>si</v>
+      </c>
+      <c r="L37" t="str">
+        <v>no</v>
+      </c>
+      <c r="M37" t="str">
+        <v>Hilo. Colores disponibles los de las fotos.</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>VE02</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Vestido Margot Hilo</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Vestidos</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E38">
+        <v>32000</v>
+      </c>
+      <c r="F38" t="str">
+        <v/>
+      </c>
+      <c r="G38">
+        <v>10</v>
+      </c>
+      <c r="H38" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I38" t="str">
+        <v>negro</v>
+      </c>
+      <c r="J38" t="str">
+        <v/>
+      </c>
+      <c r="K38" t="str">
+        <v>no</v>
+      </c>
+      <c r="L38" t="str">
+        <v>no</v>
+      </c>
+      <c r="M38" t="str">
+        <v>Importado, hilo lycra premium. Talle único.</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>VE03</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Vestido Olimpia Encaje</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Vestidos</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E39">
+        <v>23500</v>
+      </c>
+      <c r="F39" t="str">
+        <v/>
+      </c>
+      <c r="G39">
+        <v>10</v>
+      </c>
+      <c r="H39" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I39" t="str">
+        <v>negro,blanco,chocolate</v>
+      </c>
+      <c r="J39" t="str">
+        <v/>
+      </c>
+      <c r="K39" t="str">
+        <v>no</v>
+      </c>
+      <c r="L39" t="str">
+        <v>no</v>
+      </c>
+      <c r="M39" t="str">
+        <v>Encaje elastizado, con short interno. Talle único, cede a un M.</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>VE04</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Vestido Soft Corto</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Vestidos</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E40">
+        <v>16000</v>
+      </c>
+      <c r="F40" t="str">
+        <v/>
+      </c>
+      <c r="G40">
+        <v>10</v>
+      </c>
+      <c r="H40" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I40" t="str">
+        <v>negro,bordo</v>
+      </c>
+      <c r="J40" t="str">
+        <v/>
+      </c>
+      <c r="K40" t="str">
+        <v>no</v>
+      </c>
+      <c r="L40" t="str">
+        <v>no</v>
+      </c>
+      <c r="M40" t="str">
+        <v>Modal soft, busto forrado. Talle único.</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>VE05</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Vestido Algodón Lycra</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Vestidos</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E41">
+        <v>16000</v>
+      </c>
+      <c r="F41" t="str">
+        <v/>
+      </c>
+      <c r="G41">
+        <v>10</v>
+      </c>
+      <c r="H41" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I41" t="str">
+        <v>chocolate,gris,negro</v>
+      </c>
+      <c r="J41" t="str">
+        <v/>
+      </c>
+      <c r="K41" t="str">
+        <v>no</v>
+      </c>
+      <c r="L41" t="str">
+        <v>no</v>
+      </c>
+      <c r="M41" t="str">
+        <v>Algodón lycra premium. Talle único.</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>VE06</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Vestido Hilo Rayado</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Vestidos</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E42">
+        <v>26500</v>
+      </c>
+      <c r="F42" t="str">
+        <v/>
+      </c>
+      <c r="G42">
+        <v>10</v>
+      </c>
+      <c r="H42" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I42" t="str">
+        <v>celeste,amarillo,chocolate</v>
+      </c>
+      <c r="J42" t="str">
+        <v/>
+      </c>
+      <c r="K42" t="str">
+        <v>si</v>
+      </c>
+      <c r="L42" t="str">
+        <v>si</v>
+      </c>
+      <c r="M42" t="str">
+        <v>Hilo lycra premium. Talle único.</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>VE07</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Vestido Largo Básico</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Vestidos</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E43">
+        <v>19000</v>
+      </c>
+      <c r="F43" t="str">
+        <v/>
+      </c>
+      <c r="G43">
+        <v>10</v>
+      </c>
+      <c r="H43" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I43" t="str">
+        <v>negro</v>
+      </c>
+      <c r="J43" t="str">
+        <v/>
+      </c>
+      <c r="K43" t="str">
+        <v>no</v>
+      </c>
+      <c r="L43" t="str">
+        <v>no</v>
+      </c>
+      <c r="M43" t="str">
+        <v>Morley capri con tajo, busto forrado. Talle único, cede a un M.</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>VE08</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Vestido Largo Marilyn</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Vestidos</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E44">
+        <v>23500</v>
+      </c>
+      <c r="F44" t="str">
+        <v/>
+      </c>
+      <c r="G44">
+        <v>10</v>
+      </c>
+      <c r="H44" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I44" t="str">
+        <v>negro</v>
+      </c>
+      <c r="J44" t="str">
+        <v/>
+      </c>
+      <c r="K44" t="str">
+        <v>no</v>
+      </c>
+      <c r="L44" t="str">
+        <v>no</v>
+      </c>
+      <c r="M44" t="str">
+        <v>Algodón lycra premium, busto forrado, con tajo. Talle único, cede a M.</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>VE09</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Vestido Largo Puntilla</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Vestidos</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E45">
+        <v>19500</v>
+      </c>
+      <c r="F45" t="str">
+        <v/>
+      </c>
+      <c r="G45">
+        <v>10</v>
+      </c>
+      <c r="H45" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I45" t="str">
+        <v>negro</v>
+      </c>
+      <c r="J45" t="str">
+        <v/>
+      </c>
+      <c r="K45" t="str">
+        <v>no</v>
+      </c>
+      <c r="L45" t="str">
+        <v>no</v>
+      </c>
+      <c r="M45" t="str">
+        <v>Morley capri con tajo. Talle único, cede a un M.</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>VE10</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Skort Lazo Encaje</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Vestidos</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E46">
+        <v>22500</v>
+      </c>
+      <c r="F46" t="str">
+        <v/>
+      </c>
+      <c r="G46">
+        <v>10</v>
+      </c>
+      <c r="H46" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I46" t="str">
+        <v>negro</v>
+      </c>
+      <c r="J46" t="str">
+        <v/>
+      </c>
+      <c r="K46" t="str">
+        <v>no</v>
+      </c>
+      <c r="L46" t="str">
+        <v>si</v>
+      </c>
+      <c r="M46" t="str">
+        <v>Encaje elastizado con short interno. Talle único, cede a 38.</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>PA01</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Wide Leg Elastizado</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Pantalones</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E47">
+        <v>25500</v>
+      </c>
+      <c r="F47" t="str">
+        <v/>
+      </c>
+      <c r="G47">
+        <v>10</v>
+      </c>
+      <c r="H47" t="str">
+        <v>38,40,42,44,46,48</v>
+      </c>
+      <c r="I47" t="str">
+        <v>jean</v>
+      </c>
+      <c r="J47" t="str">
+        <v/>
+      </c>
+      <c r="K47" t="str">
+        <v>no</v>
+      </c>
+      <c r="L47" t="str">
+        <v>no</v>
+      </c>
+      <c r="M47" t="str">
+        <v>Jean elastizado, pierna amplia.</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>PA02</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Oxford</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Pantalones</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E48">
+        <v>25500</v>
+      </c>
+      <c r="F48" t="str">
+        <v/>
+      </c>
+      <c r="G48">
+        <v>10</v>
+      </c>
+      <c r="H48" t="str">
+        <v>38,40,42,44,46,48</v>
+      </c>
+      <c r="I48" t="str">
+        <v>negro</v>
+      </c>
+      <c r="J48" t="str">
+        <v>aika-09.jpg</v>
+      </c>
+      <c r="K48" t="str">
+        <v>si</v>
+      </c>
+      <c r="L48" t="str">
+        <v>no</v>
+      </c>
+      <c r="M48" t="str">
+        <v>Lycra importada, cintura en V y línea al costado.</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>PA03</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Wide Leg con Rotura</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Pantalones</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E49">
+        <v>26500</v>
+      </c>
+      <c r="F49" t="str">
+        <v/>
+      </c>
+      <c r="G49">
+        <v>10</v>
+      </c>
+      <c r="H49" t="str">
+        <v>36,38</v>
+      </c>
+      <c r="I49" t="str">
+        <v>jean</v>
+      </c>
+      <c r="J49" t="str">
+        <v/>
+      </c>
+      <c r="K49" t="str">
+        <v>no</v>
+      </c>
+      <c r="L49" t="str">
+        <v>no</v>
+      </c>
+      <c r="M49" t="str">
+        <v>Jean rígido con roturas.</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>PA04</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Pollera Polly</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Pantalones</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E50">
+        <v>27000</v>
+      </c>
+      <c r="F50" t="str">
+        <v/>
+      </c>
+      <c r="G50">
+        <v>10</v>
+      </c>
+      <c r="H50" t="str">
+        <v>36,38,40,42,44,46</v>
+      </c>
+      <c r="I50" t="str">
+        <v>jean</v>
+      </c>
+      <c r="J50" t="str">
+        <v/>
+      </c>
+      <c r="K50" t="str">
+        <v>no</v>
+      </c>
+      <c r="L50" t="str">
+        <v>no</v>
+      </c>
+      <c r="M50" t="str">
+        <v>Jean rígido.</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>PA05</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Baggy Camuflado</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Pantalones</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E51">
+        <v>32000</v>
+      </c>
+      <c r="F51" t="str">
+        <v/>
+      </c>
+      <c r="G51">
+        <v>10</v>
+      </c>
+      <c r="H51" t="str">
+        <v>36,38,40,42,44,46</v>
+      </c>
+      <c r="I51" t="str">
+        <v>verde</v>
+      </c>
+      <c r="J51" t="str">
+        <v/>
+      </c>
+      <c r="K51" t="str">
+        <v>no</v>
+      </c>
+      <c r="L51" t="str">
+        <v>no</v>
+      </c>
+      <c r="M51" t="str">
+        <v>Rígido, estampa camuflada.</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>PA06</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Palazo Sastrero con Cinto</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Pantalones</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E52">
+        <v>23500</v>
+      </c>
+      <c r="F52" t="str">
+        <v/>
+      </c>
+      <c r="G52">
+        <v>10</v>
+      </c>
+      <c r="H52" t="str">
+        <v>2,3,4,5</v>
+      </c>
+      <c r="I52" t="str">
+        <v>negro</v>
+      </c>
+      <c r="J52" t="str">
+        <v/>
+      </c>
+      <c r="K52" t="str">
+        <v>no</v>
+      </c>
+      <c r="L52" t="str">
+        <v>no</v>
+      </c>
+      <c r="M52" t="str">
+        <v>Creep sastrero con cinto.</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>PA07</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Oxford London</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Pantalones</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E53">
+        <v>21000</v>
+      </c>
+      <c r="F53" t="str">
+        <v/>
+      </c>
+      <c r="G53">
+        <v>10</v>
+      </c>
+      <c r="H53" t="str">
+        <v>M (36/38),G (40),GG (42/44)</v>
+      </c>
+      <c r="I53" t="str">
+        <v>negro</v>
+      </c>
+      <c r="J53" t="str">
+        <v/>
+      </c>
+      <c r="K53" t="str">
+        <v>no</v>
+      </c>
+      <c r="L53" t="str">
+        <v>no</v>
+      </c>
+      <c r="M53" t="str">
+        <v>Oxford clásico.</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>PA08</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Baggy Batik</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Pantalones</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E54">
+        <v>21500</v>
+      </c>
+      <c r="F54" t="str">
+        <v/>
+      </c>
+      <c r="G54">
+        <v>10</v>
+      </c>
+      <c r="H54" t="str">
+        <v>2 (38),3 (40),4 (42),5 (44/46)</v>
+      </c>
+      <c r="I54" t="str">
+        <v>gris</v>
+      </c>
+      <c r="J54" t="str">
+        <v>aika-04.jpg</v>
+      </c>
+      <c r="K54" t="str">
+        <v>si</v>
+      </c>
+      <c r="L54" t="str">
+        <v>no</v>
+      </c>
+      <c r="M54" t="str">
+        <v>Tela rústica batik, bolsillos laterales y tanca ajustable.</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>PA09</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Pantalón Linora</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Pantalones</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E55">
+        <v>22000</v>
+      </c>
+      <c r="F55" t="str">
+        <v/>
+      </c>
+      <c r="G55">
+        <v>10</v>
+      </c>
+      <c r="H55" t="str">
+        <v>2 (38),3 (40),4 (42),5 (44)</v>
+      </c>
+      <c r="I55" t="str">
+        <v>beige,celeste,verde,negro</v>
+      </c>
+      <c r="J55" t="str">
+        <v/>
+      </c>
+      <c r="K55" t="str">
+        <v>no</v>
+      </c>
+      <c r="L55" t="str">
+        <v>no</v>
+      </c>
+      <c r="M55" t="str">
+        <v>Sin cambio.</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>SH01</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Short Tira Cruzado</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Shorts</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E56">
+        <v>23000</v>
+      </c>
+      <c r="F56" t="str">
+        <v/>
+      </c>
+      <c r="G56">
+        <v>10</v>
+      </c>
+      <c r="H56" t="str">
+        <v>36,38,40,42,44,46</v>
+      </c>
+      <c r="I56" t="str">
+        <v>jean</v>
+      </c>
+      <c r="J56" t="str">
+        <v/>
+      </c>
+      <c r="K56" t="str">
+        <v>no</v>
+      </c>
+      <c r="L56" t="str">
+        <v>no</v>
+      </c>
+      <c r="M56" t="str">
+        <v>Jean con tiras cruzadas.</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>SH02</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Short Botón</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Shorts</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E57">
+        <v>23000</v>
+      </c>
+      <c r="F57" t="str">
+        <v/>
+      </c>
+      <c r="G57">
+        <v>10</v>
+      </c>
+      <c r="H57" t="str">
+        <v>36,38,40,42,44,46</v>
+      </c>
+      <c r="I57" t="str">
+        <v>jean</v>
+      </c>
+      <c r="J57" t="str">
+        <v/>
+      </c>
+      <c r="K57" t="str">
+        <v>no</v>
+      </c>
+      <c r="L57" t="str">
+        <v>no</v>
+      </c>
+      <c r="M57" t="str">
+        <v>Jean con botones.</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>SH03</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Bermuda Clasic</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Shorts</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E58">
+        <v>24000</v>
+      </c>
+      <c r="F58" t="str">
+        <v/>
+      </c>
+      <c r="G58">
+        <v>10</v>
+      </c>
+      <c r="H58" t="str">
+        <v>36,38,40,42,44,46</v>
+      </c>
+      <c r="I58" t="str">
+        <v>jean</v>
+      </c>
+      <c r="J58" t="str">
+        <v/>
+      </c>
+      <c r="K58" t="str">
+        <v>no</v>
+      </c>
+      <c r="L58" t="str">
+        <v>no</v>
+      </c>
+      <c r="M58" t="str">
+        <v>Bolsillos traseros.</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>SH04</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Short Pollera Napoleón</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Shorts</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E59">
+        <v>25000</v>
+      </c>
+      <c r="F59" t="str">
+        <v/>
+      </c>
+      <c r="G59">
+        <v>10</v>
+      </c>
+      <c r="H59" t="str">
+        <v>36,38,40,42,44,46</v>
+      </c>
+      <c r="I59" t="str">
+        <v>celeste,azul</v>
+      </c>
+      <c r="J59" t="str">
+        <v/>
+      </c>
+      <c r="K59" t="str">
+        <v>no</v>
+      </c>
+      <c r="L59" t="str">
+        <v>no</v>
+      </c>
+      <c r="M59" t="str">
+        <v>Jean rígido con bolsillo.</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>SH05</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Short Creep con Cinto</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Shorts</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E60">
+        <v>20000</v>
+      </c>
+      <c r="F60" t="str">
+        <v/>
+      </c>
+      <c r="G60">
+        <v>10</v>
+      </c>
+      <c r="H60" t="str">
+        <v>2,3,4,5</v>
+      </c>
+      <c r="I60" t="str">
+        <v>chocolate,negro,camel</v>
+      </c>
+      <c r="J60" t="str">
+        <v>aika-07.jpg</v>
+      </c>
+      <c r="K60" t="str">
+        <v>si</v>
+      </c>
+      <c r="L60" t="str">
+        <v>no</v>
+      </c>
+      <c r="M60" t="str">
+        <v>Creep sastrero con cinto.</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>SH06</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Short Fit</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Shorts</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E61">
+        <v>18000</v>
+      </c>
+      <c r="F61" t="str">
+        <v/>
+      </c>
+      <c r="G61">
+        <v>10</v>
+      </c>
+      <c r="H61" t="str">
+        <v>S/M (38/40),L/XL (42/44)</v>
+      </c>
+      <c r="I61" t="str">
+        <v>chocolate,bordo,azul,topo,camel,celeste,negro</v>
+      </c>
+      <c r="J61" t="str">
+        <v/>
+      </c>
+      <c r="K61" t="str">
+        <v>no</v>
+      </c>
+      <c r="L61" t="str">
+        <v>no</v>
+      </c>
+      <c r="M61" t="str">
+        <v>S/M: choco, bordo, azul eléctrico, topo, camel. L/XL: celeste, negro, azul eléctrico, gris topo. Sin cambio.</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>AB01</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Campera Rústica Corta</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Abrigos</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E62">
+        <v>26000</v>
+      </c>
+      <c r="F62" t="str">
+        <v/>
+      </c>
+      <c r="G62">
+        <v>10</v>
+      </c>
+      <c r="H62" t="str">
+        <v>Único</v>
+      </c>
+      <c r="I62" t="str">
+        <v>negro</v>
+      </c>
+      <c r="J62" t="str">
+        <v/>
+      </c>
+      <c r="K62" t="str">
+        <v>no</v>
+      </c>
+      <c r="L62" t="str">
+        <v>no</v>
+      </c>
+      <c r="M62" t="str">
+        <v>Campera de tela rústica, corta.</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>AB02</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Cardigan Calado Hilo</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Abrigos</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E63">
+        <v>29000</v>
+      </c>
+      <c r="F63" t="str">
+        <v/>
+      </c>
+      <c r="G63">
+        <v>10</v>
+      </c>
+      <c r="H63" t="str">
+        <v>Único (hasta L)</v>
+      </c>
+      <c r="I63" t="str">
+        <v>negro,marron,chocolate</v>
+      </c>
+      <c r="J63" t="str">
+        <v/>
+      </c>
+      <c r="K63" t="str">
+        <v>no</v>
+      </c>
+      <c r="L63" t="str">
+        <v>no</v>
+      </c>
+      <c r="M63" t="str">
+        <v>Hilo de algodón premium (hilado de verano). Modelo oversize.</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>AB03</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Campera Oversize Tencel</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Abrigos</v>
+      </c>
+      <c r="D64" t="str">
+        <v>Mujer</v>
+      </c>
+      <c r="E64">
+        <v>35500</v>
+      </c>
+      <c r="F64" t="str">
+        <v/>
+      </c>
+      <c r="G64">
+        <v>10</v>
+      </c>
+      <c r="H64" t="str">
+        <v>Único (aprox. L/XL)</v>
+      </c>
+      <c r="I64" t="str">
+        <v>negro,crudo,chocolate</v>
+      </c>
+      <c r="J64" t="str">
+        <v/>
+      </c>
+      <c r="K64" t="str">
+        <v>no</v>
+      </c>
+      <c r="L64" t="str">
+        <v>no</v>
+      </c>
+      <c r="M64" t="str">
+        <v>Tencel símil lino, modelo oversize (amplio).</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M64"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C9"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -856,7 +3070,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Enteritos</v>
+        <v>Bodys y catsuits</v>
       </c>
       <c r="B2" t="str">
         <v>vestido</v>
@@ -878,10 +3092,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Pantalones</v>
+        <v>Musculosas</v>
       </c>
       <c r="B4" t="str">
-        <v>pantalon</v>
+        <v>remera</v>
       </c>
       <c r="C4">
         <v>3</v>
@@ -889,10 +3103,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Shorts</v>
+        <v>Remeras</v>
       </c>
       <c r="B5" t="str">
-        <v>pantalon</v>
+        <v>remera</v>
       </c>
       <c r="C5">
         <v>4</v>
@@ -909,9 +3123,42 @@
         <v>5</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Pantalones</v>
+      </c>
+      <c r="B7" t="str">
+        <v>pantalon</v>
+      </c>
+      <c r="C7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Shorts</v>
+      </c>
+      <c r="B8" t="str">
+        <v>pantalon</v>
+      </c>
+      <c r="C8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Abrigos</v>
+      </c>
+      <c r="B9" t="str">
+        <v>blazer</v>
+      </c>
+      <c r="C9">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C9"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fotos reales del catálogo (81, WebP 900x1125) asignadas a cada producto
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/aika.xlsx
+++ b/data/aika.xlsx
@@ -484,10 +484,10 @@
         <v>S/M (38/40),L/XL (42/44)</v>
       </c>
       <c r="I2" t="str">
-        <v>rosa,bordo,rosa claro,gris azulado,azul marino,verde,negro,azul,celeste</v>
+        <v>rosa claro,rosa,bordo,negro,gris azulado,azul marino,verde,celeste,azul</v>
       </c>
       <c r="J2" t="str">
-        <v>aika-10.jpg,aika-11.jpg,aika-12.jpg,aika-13.jpg,aika-14.jpg,aika-15.jpg,aika-16.jpg,aika-17.jpg,aika-18.jpg,aika-19.jpg</v>
+        <v>cs01-1.webp,cs01-2.webp,cs01-3.webp,cs01-4.webp,cs01-5.webp,cs01-6.webp,cs01-7.webp,cs01-8.webp,cs01-9.webp</v>
       </c>
       <c r="K2" t="str">
         <v>si</v>
@@ -528,7 +528,7 @@
         <v>negro,gris,blanco,chocolate,rosa,azul,rojo</v>
       </c>
       <c r="J3" t="str">
-        <v/>
+        <v>cs02-1.webp</v>
       </c>
       <c r="K3" t="str">
         <v>no</v>
@@ -569,7 +569,7 @@
         <v>negro</v>
       </c>
       <c r="J4" t="str">
-        <v/>
+        <v>cs03-1.webp</v>
       </c>
       <c r="K4" t="str">
         <v>no</v>
@@ -607,10 +607,10 @@
         <v>Único</v>
       </c>
       <c r="I5" t="str">
-        <v>negro</v>
+        <v>chocolate,negro,blanco</v>
       </c>
       <c r="J5" t="str">
-        <v/>
+        <v>bo01-1.webp</v>
       </c>
       <c r="K5" t="str">
         <v>no</v>
@@ -651,7 +651,7 @@
         <v>negro</v>
       </c>
       <c r="J6" t="str">
-        <v/>
+        <v>bo02-1.webp</v>
       </c>
       <c r="K6" t="str">
         <v>no</v>
@@ -692,7 +692,7 @@
         <v>negro</v>
       </c>
       <c r="J7" t="str">
-        <v/>
+        <v>bo03-1.webp</v>
       </c>
       <c r="K7" t="str">
         <v>no</v>
@@ -733,7 +733,7 @@
         <v>negro</v>
       </c>
       <c r="J8" t="str">
-        <v/>
+        <v>bo04-1.webp</v>
       </c>
       <c r="K8" t="str">
         <v>no</v>
@@ -774,7 +774,7 @@
         <v>negro,topo,gris,blanco,chocolate</v>
       </c>
       <c r="J9" t="str">
-        <v>aika-01.jpg</v>
+        <v>tp01-1.webp</v>
       </c>
       <c r="K9" t="str">
         <v>si</v>
@@ -815,7 +815,7 @@
         <v>negro,blanco,chocolate</v>
       </c>
       <c r="J10" t="str">
-        <v/>
+        <v>tp02-1.webp</v>
       </c>
       <c r="K10" t="str">
         <v>no</v>
@@ -856,7 +856,7 @@
         <v>negro,blanco,celeste,chocolate,gris</v>
       </c>
       <c r="J11" t="str">
-        <v/>
+        <v>tp03-1.webp</v>
       </c>
       <c r="K11" t="str">
         <v>no</v>
@@ -897,7 +897,7 @@
         <v>negro,blanco,chocolate</v>
       </c>
       <c r="J12" t="str">
-        <v/>
+        <v>tp04-1.webp</v>
       </c>
       <c r="K12" t="str">
         <v>no</v>
@@ -938,7 +938,7 @@
         <v>negro,blanco</v>
       </c>
       <c r="J13" t="str">
-        <v/>
+        <v>tp05-1.webp,tp05-2.webp</v>
       </c>
       <c r="K13" t="str">
         <v>no</v>
@@ -979,7 +979,7 @@
         <v>blanco,negro,chocolate</v>
       </c>
       <c r="J14" t="str">
-        <v/>
+        <v>tp06-1.webp,tp06-2.webp</v>
       </c>
       <c r="K14" t="str">
         <v>no</v>
@@ -1020,7 +1020,7 @@
         <v>negro,chocolate,blanco</v>
       </c>
       <c r="J15" t="str">
-        <v/>
+        <v>tp07-1.webp</v>
       </c>
       <c r="K15" t="str">
         <v>no</v>
@@ -1061,7 +1061,7 @@
         <v>negro</v>
       </c>
       <c r="J16" t="str">
-        <v/>
+        <v>tp08-1.webp</v>
       </c>
       <c r="K16" t="str">
         <v>si</v>
@@ -1102,7 +1102,7 @@
         <v>blanco,negro,gris,rosa claro,celeste,marron</v>
       </c>
       <c r="J17" t="str">
-        <v>aika-05.jpg</v>
+        <v>mu01-1.webp</v>
       </c>
       <c r="K17" t="str">
         <v>si</v>
@@ -1143,7 +1143,7 @@
         <v>rosa,gris,negro,blanco,marron</v>
       </c>
       <c r="J18" t="str">
-        <v>aika-08.jpg</v>
+        <v>mu02-1.webp</v>
       </c>
       <c r="K18" t="str">
         <v>no</v>
@@ -1184,7 +1184,7 @@
         <v>chocolate,blanco,negro</v>
       </c>
       <c r="J19" t="str">
-        <v>aika-02.jpg</v>
+        <v>mu03-1.webp</v>
       </c>
       <c r="K19" t="str">
         <v>no</v>
@@ -1225,7 +1225,7 @@
         <v>celeste,rosa</v>
       </c>
       <c r="J20" t="str">
-        <v>aika-03.jpg</v>
+        <v>mu04-1.webp</v>
       </c>
       <c r="K20" t="str">
         <v>no</v>
@@ -1266,7 +1266,7 @@
         <v>chocolate,negro</v>
       </c>
       <c r="J21" t="str">
-        <v/>
+        <v>mu05-1.webp</v>
       </c>
       <c r="K21" t="str">
         <v>no</v>
@@ -1307,7 +1307,7 @@
         <v>negro</v>
       </c>
       <c r="J22" t="str">
-        <v/>
+        <v>mu06-1.webp</v>
       </c>
       <c r="K22" t="str">
         <v>no</v>
@@ -1348,7 +1348,7 @@
         <v>negro,blanco,chocolate</v>
       </c>
       <c r="J23" t="str">
-        <v/>
+        <v>mu07-1.webp,mu07-2.webp</v>
       </c>
       <c r="K23" t="str">
         <v>no</v>
@@ -1389,7 +1389,7 @@
         <v>frambuesa,blanco,chocolate,negro</v>
       </c>
       <c r="J24" t="str">
-        <v/>
+        <v>mu08-1.webp</v>
       </c>
       <c r="K24" t="str">
         <v>no</v>
@@ -1430,7 +1430,7 @@
         <v>negro</v>
       </c>
       <c r="J25" t="str">
-        <v/>
+        <v>re01-1.webp</v>
       </c>
       <c r="K25" t="str">
         <v>no</v>
@@ -1471,7 +1471,7 @@
         <v>negro</v>
       </c>
       <c r="J26" t="str">
-        <v/>
+        <v>re02-1.webp</v>
       </c>
       <c r="K26" t="str">
         <v>no</v>
@@ -1512,7 +1512,7 @@
         <v>chocolate,blanco,negro,bordo</v>
       </c>
       <c r="J27" t="str">
-        <v/>
+        <v>re03-1.webp</v>
       </c>
       <c r="K27" t="str">
         <v>si</v>
@@ -1553,7 +1553,7 @@
         <v>negro,blanco,topo,chocolate,marron</v>
       </c>
       <c r="J28" t="str">
-        <v/>
+        <v>re04-1.webp</v>
       </c>
       <c r="K28" t="str">
         <v>no</v>
@@ -1594,7 +1594,7 @@
         <v>chocolate,blanco,negro</v>
       </c>
       <c r="J29" t="str">
-        <v/>
+        <v>re05-1.webp</v>
       </c>
       <c r="K29" t="str">
         <v>no</v>
@@ -1635,7 +1635,7 @@
         <v>negro,blanco,chocolate</v>
       </c>
       <c r="J30" t="str">
-        <v/>
+        <v>re06-1.webp</v>
       </c>
       <c r="K30" t="str">
         <v>no</v>
@@ -1676,7 +1676,7 @@
         <v>negro,gris,blanco,chocolate</v>
       </c>
       <c r="J31" t="str">
-        <v/>
+        <v>re07-1.webp</v>
       </c>
       <c r="K31" t="str">
         <v>no</v>
@@ -1717,7 +1717,7 @@
         <v>azul,negro,chocolate,rojo</v>
       </c>
       <c r="J32" t="str">
-        <v/>
+        <v>re08-1.webp</v>
       </c>
       <c r="K32" t="str">
         <v>no</v>
@@ -1758,7 +1758,7 @@
         <v>blanco</v>
       </c>
       <c r="J33" t="str">
-        <v/>
+        <v>re09-1.webp</v>
       </c>
       <c r="K33" t="str">
         <v>no</v>
@@ -1799,7 +1799,7 @@
         <v>negro</v>
       </c>
       <c r="J34" t="str">
-        <v/>
+        <v>re10-1.webp</v>
       </c>
       <c r="K34" t="str">
         <v>no</v>
@@ -1840,7 +1840,7 @@
         <v>chocolate,blanco,negro</v>
       </c>
       <c r="J35" t="str">
-        <v/>
+        <v>re11-1.webp</v>
       </c>
       <c r="K35" t="str">
         <v>no</v>
@@ -1881,7 +1881,7 @@
         <v>crudo,negro,beige,azul,verde</v>
       </c>
       <c r="J36" t="str">
-        <v/>
+        <v>re12-1.webp</v>
       </c>
       <c r="K36" t="str">
         <v>no</v>
@@ -1922,7 +1922,7 @@
         <v>crudo,chocolate,blanco,negro</v>
       </c>
       <c r="J37" t="str">
-        <v>aika-06.jpg</v>
+        <v>ve01-1.webp</v>
       </c>
       <c r="K37" t="str">
         <v>si</v>
@@ -1963,7 +1963,7 @@
         <v>negro</v>
       </c>
       <c r="J38" t="str">
-        <v/>
+        <v>ve02-1.webp</v>
       </c>
       <c r="K38" t="str">
         <v>no</v>
@@ -2004,7 +2004,7 @@
         <v>negro,blanco,chocolate</v>
       </c>
       <c r="J39" t="str">
-        <v/>
+        <v>ve03-1.webp,ve03-2.webp</v>
       </c>
       <c r="K39" t="str">
         <v>no</v>
@@ -2045,7 +2045,7 @@
         <v>negro,bordo</v>
       </c>
       <c r="J40" t="str">
-        <v/>
+        <v>ve04-1.webp</v>
       </c>
       <c r="K40" t="str">
         <v>no</v>
@@ -2086,7 +2086,7 @@
         <v>chocolate,gris,negro</v>
       </c>
       <c r="J41" t="str">
-        <v/>
+        <v>ve05-1.webp</v>
       </c>
       <c r="K41" t="str">
         <v>no</v>
@@ -2127,7 +2127,7 @@
         <v>celeste,amarillo,chocolate</v>
       </c>
       <c r="J42" t="str">
-        <v/>
+        <v>ve06-1.webp,ve06-2.webp</v>
       </c>
       <c r="K42" t="str">
         <v>si</v>
@@ -2168,7 +2168,7 @@
         <v>negro</v>
       </c>
       <c r="J43" t="str">
-        <v/>
+        <v>ve07-1.webp</v>
       </c>
       <c r="K43" t="str">
         <v>no</v>
@@ -2209,7 +2209,7 @@
         <v>negro</v>
       </c>
       <c r="J44" t="str">
-        <v/>
+        <v>ve08-1.webp,ve08-2.webp</v>
       </c>
       <c r="K44" t="str">
         <v>no</v>
@@ -2250,7 +2250,7 @@
         <v>negro</v>
       </c>
       <c r="J45" t="str">
-        <v/>
+        <v>ve09-1.webp</v>
       </c>
       <c r="K45" t="str">
         <v>no</v>
@@ -2291,7 +2291,7 @@
         <v>negro</v>
       </c>
       <c r="J46" t="str">
-        <v/>
+        <v>ve10-1.webp</v>
       </c>
       <c r="K46" t="str">
         <v>no</v>
@@ -2332,7 +2332,7 @@
         <v>jean</v>
       </c>
       <c r="J47" t="str">
-        <v/>
+        <v>pa01-1.webp,pa01-2.webp</v>
       </c>
       <c r="K47" t="str">
         <v>no</v>
@@ -2370,10 +2370,10 @@
         <v>38,40,42,44,46,48</v>
       </c>
       <c r="I48" t="str">
-        <v>negro</v>
+        <v>jean</v>
       </c>
       <c r="J48" t="str">
-        <v>aika-09.jpg</v>
+        <v>pa02-1.webp</v>
       </c>
       <c r="K48" t="str">
         <v>si</v>
@@ -2382,7 +2382,7 @@
         <v>no</v>
       </c>
       <c r="M48" t="str">
-        <v>Lycra importada, cintura en V y línea al costado.</v>
+        <v>Jean elastizado, corte oxford.</v>
       </c>
     </row>
     <row r="49">
@@ -2414,7 +2414,7 @@
         <v>jean</v>
       </c>
       <c r="J49" t="str">
-        <v/>
+        <v>pa03-1.webp</v>
       </c>
       <c r="K49" t="str">
         <v>no</v>
@@ -2455,7 +2455,7 @@
         <v>jean</v>
       </c>
       <c r="J50" t="str">
-        <v/>
+        <v>pa04-1.webp</v>
       </c>
       <c r="K50" t="str">
         <v>no</v>
@@ -2496,7 +2496,7 @@
         <v>verde</v>
       </c>
       <c r="J51" t="str">
-        <v/>
+        <v>pa05-1.webp</v>
       </c>
       <c r="K51" t="str">
         <v>no</v>
@@ -2537,7 +2537,7 @@
         <v>negro</v>
       </c>
       <c r="J52" t="str">
-        <v/>
+        <v>pa06-1.webp</v>
       </c>
       <c r="K52" t="str">
         <v>no</v>
@@ -2578,7 +2578,7 @@
         <v>negro</v>
       </c>
       <c r="J53" t="str">
-        <v/>
+        <v>pa07-1.webp</v>
       </c>
       <c r="K53" t="str">
         <v>no</v>
@@ -2619,7 +2619,7 @@
         <v>gris</v>
       </c>
       <c r="J54" t="str">
-        <v>aika-04.jpg</v>
+        <v>pa08-1.webp</v>
       </c>
       <c r="K54" t="str">
         <v>si</v>
@@ -2660,7 +2660,7 @@
         <v>beige,celeste,verde,negro</v>
       </c>
       <c r="J55" t="str">
-        <v/>
+        <v>pa09-1.webp</v>
       </c>
       <c r="K55" t="str">
         <v>no</v>
@@ -2701,7 +2701,7 @@
         <v>jean</v>
       </c>
       <c r="J56" t="str">
-        <v/>
+        <v>sh01-1.webp</v>
       </c>
       <c r="K56" t="str">
         <v>no</v>
@@ -2742,7 +2742,7 @@
         <v>jean</v>
       </c>
       <c r="J57" t="str">
-        <v/>
+        <v>sh02-1.webp</v>
       </c>
       <c r="K57" t="str">
         <v>no</v>
@@ -2783,7 +2783,7 @@
         <v>jean</v>
       </c>
       <c r="J58" t="str">
-        <v/>
+        <v>sh03-1.webp</v>
       </c>
       <c r="K58" t="str">
         <v>no</v>
@@ -2824,7 +2824,7 @@
         <v>celeste,azul</v>
       </c>
       <c r="J59" t="str">
-        <v/>
+        <v>sh04-1.webp,sh04-2.webp</v>
       </c>
       <c r="K59" t="str">
         <v>no</v>
@@ -2865,7 +2865,7 @@
         <v>chocolate,negro,camel</v>
       </c>
       <c r="J60" t="str">
-        <v>aika-07.jpg</v>
+        <v>sh05-1.webp</v>
       </c>
       <c r="K60" t="str">
         <v>si</v>
@@ -2906,7 +2906,7 @@
         <v>chocolate,bordo,azul,topo,camel,celeste,negro</v>
       </c>
       <c r="J61" t="str">
-        <v/>
+        <v>sh06-1.webp</v>
       </c>
       <c r="K61" t="str">
         <v>no</v>
@@ -2947,7 +2947,7 @@
         <v>negro</v>
       </c>
       <c r="J62" t="str">
-        <v/>
+        <v>ab01-1.webp,ab01-2.webp,ab01-3.webp</v>
       </c>
       <c r="K62" t="str">
         <v>no</v>
@@ -2988,7 +2988,7 @@
         <v>negro,marron,chocolate</v>
       </c>
       <c r="J63" t="str">
-        <v/>
+        <v>ab02-1.webp</v>
       </c>
       <c r="K63" t="str">
         <v>no</v>
@@ -3029,7 +3029,7 @@
         <v>negro,crudo,chocolate</v>
       </c>
       <c r="J64" t="str">
-        <v/>
+        <v>ab03-1.webp</v>
       </c>
       <c r="K64" t="str">
         <v>no</v>
@@ -3272,7 +3272,7 @@
         <v>promo_imagen</v>
       </c>
       <c r="B13" t="str">
-        <v>/productos/aika-07.jpg</v>
+        <v>sh05-1.webp</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Portada con foto optimizada local y movimiento de cámara leve; bolsa en el burger; WhatsApp flotante oculto en la ficha; el vuelo se suelta al scrollear
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/aika.xlsx
+++ b/data/aika.xlsx
@@ -401,21 +401,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M64"/>
-  <cols>
-    <col min="1" max="1" width="7.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="9.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="7" max="7" width="7.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="26.83203125" customWidth="1"/>
-    <col min="10" max="10" width="40.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="7.83203125" customWidth="1"/>
-    <col min="13" max="13" width="50.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3051,11 +3036,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C9"/>
-  <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="7.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3166,10 +3146,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B13"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="60.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3248,7 +3224,7 @@
         <v>hero_imagen</v>
       </c>
       <c r="B10" t="str">
-        <v>https://images.unsplash.com/photo-1515886657613-9f3515b0c78f?w=800&amp;q=80&amp;auto=format&amp;fit=crop</v>
+        <v>/hero-1515886657613.webp</v>
       </c>
     </row>
     <row r="11">
@@ -3285,9 +3261,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A9"/>
-  <cols>
-    <col min="1" max="1" width="110.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>